<commit_message>
Reorganize codebase into packages and add new features
- Restructured into packages: data/, compute_momentum/, comomentum/, fama_macbeth/, adjusted_momentum/, streamlit_app/
- Added sys.path guards to all subfolder modules for standalone execution
- New: comomentum time-series plot (plot_comom_time_series.py)
- New: market variables MRET/MVOL (data/market_variables.py)
- New: summary statistics table replicating Lou & Polk Table I (comomentum/summary_statistics_table.py)
- New: Streamlit app with Data Loading, Raw Data Preview, and Momentum Factor pages
- Updated all imports in momentum_strategy.py and cross-module references
- Added requirements.txt
</commit_message>
<xml_diff>
--- a/output_data/ff3_residuals.xlsx
+++ b/output_data/ff3_residuals.xlsx
@@ -19,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -36,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,12 +47,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,12 +431,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
@@ -701,869 +713,869 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Acadia Realty Trust</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>AerCap Holdings NV</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Allegheny Technologies Incorporated</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Alliance Data Systems Corporation</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Ambac Financial Group, Inc.</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>American Airlines Group, Inc.</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>American Assets Trust, Inc.</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Apache Corporation</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Apollo Commercial Real Estate Finance, Inc.</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Argo Group International Holdings, Ltd.</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Assured Guaranty Ltd.</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Avnet, Inc.</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Hope Bancorp, Inc.</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Belden Inc.</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>BGC Partners, Inc. Class A</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Blackbaud, Inc.</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>bluebird bio, Inc.</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Boeing Company</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Cardiovascular Systems, Inc.</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Cardtronics plc Class A</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Perdoceo Education Corporation</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Carnival Corporation</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Carpenter Technology Corporation</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Chimera Investment Corporation</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Cinemark Holdings, Inc.</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Citigroup Inc.</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Coherent, Inc.</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Columbia Property Trust, Inc.</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>DXC Technology Co.</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Concho Resources Inc.</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>ConocoPhillips</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Continental Resources, Inc.</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>CoreCivic, Inc.</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Coty Inc. Class A</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Credit Acceptance Corporation</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>CVR Energy, Inc.</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>LivaNova Plc</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Delek US Holdings Inc</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Delta Air Lines, Inc.</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>Deluxe Corporation</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>Devon Energy Corporation</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>Diamondback Energy, Inc.</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>DiamondRock Hospitality Company</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>Douglas Dynamics, Inc.</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>Dril-Quip, Inc.</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>EchoStar Corporation Class A</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>Empire State Realty Trust, Inc. Class A</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>Enanta Pharmaceuticals, Inc.</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>EOG Resources, Inc.</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>Epizyme, Inc.</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>EPR Properties</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>Exxon Mobil Corporation</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BB1" s="1" t="inlineStr">
         <is>
           <t>Federal Realty Investment Trust</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BC1" s="1" t="inlineStr">
         <is>
           <t>First Commonwealth Financial Corporation</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BD1" s="1" t="inlineStr">
         <is>
           <t>First Financial Bancorp.</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>First Midwest Bancorp, Inc.</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>FirstEnergy Corp.</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BG1" s="1" t="inlineStr">
         <is>
           <t>Flowserve Corporation</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BH1" s="1" t="inlineStr">
         <is>
           <t>Fresh Del Monte Produce Inc.</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BI1" s="1" t="inlineStr">
         <is>
           <t>GEO Group Inc</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BJ1" s="1" t="inlineStr">
         <is>
           <t>Golar LNG Limited</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BK1" s="1" t="inlineStr">
         <is>
           <t>Goodyear Tire &amp; Rubber Company</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BL1" s="1" t="inlineStr">
         <is>
           <t>Graham Holdings Co.</t>
         </is>
       </c>
-      <c r="BM1" t="inlineStr">
+      <c r="BM1" s="1" t="inlineStr">
         <is>
           <t>Halliburton Company</t>
         </is>
       </c>
-      <c r="BN1" t="inlineStr">
+      <c r="BN1" s="1" t="inlineStr">
         <is>
           <t>Hancock Whitney Corporation</t>
         </is>
       </c>
-      <c r="BO1" t="inlineStr">
+      <c r="BO1" s="1" t="inlineStr">
         <is>
           <t>Helmerich &amp; Payne, Inc.</t>
         </is>
       </c>
-      <c r="BP1" t="inlineStr">
+      <c r="BP1" s="1" t="inlineStr">
         <is>
           <t>HollyFrontier Corporation</t>
         </is>
       </c>
-      <c r="BQ1" t="inlineStr">
+      <c r="BQ1" s="1" t="inlineStr">
         <is>
           <t>Service Properties Trust</t>
         </is>
       </c>
-      <c r="BR1" t="inlineStr">
+      <c r="BR1" s="1" t="inlineStr">
         <is>
           <t>Howard Hughes Corporation</t>
         </is>
       </c>
-      <c r="BS1" t="inlineStr">
+      <c r="BS1" s="1" t="inlineStr">
         <is>
           <t>Huntington Ingalls Industries, Inc.</t>
         </is>
       </c>
-      <c r="BT1" t="inlineStr">
+      <c r="BT1" s="1" t="inlineStr">
         <is>
           <t>Huron Consulting Group Inc.</t>
         </is>
       </c>
-      <c r="BU1" t="inlineStr">
+      <c r="BU1" s="1" t="inlineStr">
         <is>
           <t>Inogen, Inc.</t>
         </is>
       </c>
-      <c r="BV1" t="inlineStr">
+      <c r="BV1" s="1" t="inlineStr">
         <is>
           <t>Intercept Pharmaceuticals, Inc.</t>
         </is>
       </c>
-      <c r="BW1" t="inlineStr">
+      <c r="BW1" s="1" t="inlineStr">
         <is>
           <t>Intra-Cellular Therapies, Inc.</t>
         </is>
       </c>
-      <c r="BX1" t="inlineStr">
+      <c r="BX1" s="1" t="inlineStr">
         <is>
           <t>Kaiser Aluminum Corporation</t>
         </is>
       </c>
-      <c r="BY1" t="inlineStr">
+      <c r="BY1" s="1" t="inlineStr">
         <is>
           <t>Kohls Corporation</t>
         </is>
       </c>
-      <c r="BZ1" t="inlineStr">
+      <c r="BZ1" s="1" t="inlineStr">
         <is>
           <t>M&amp;T Bank Corporation</t>
         </is>
       </c>
-      <c r="CA1" t="inlineStr">
+      <c r="CA1" s="1" t="inlineStr">
         <is>
           <t>Macerich Company</t>
         </is>
       </c>
-      <c r="CB1" t="inlineStr">
+      <c r="CB1" s="1" t="inlineStr">
         <is>
           <t>Mack-Cali Realty Corporation</t>
         </is>
       </c>
-      <c r="CC1" t="inlineStr">
+      <c r="CC1" s="1" t="inlineStr">
         <is>
           <t>Macquarie Infrastructure Corporation</t>
         </is>
       </c>
-      <c r="CD1" t="inlineStr">
+      <c r="CD1" s="1" t="inlineStr">
         <is>
           <t>Macys Inc</t>
         </is>
       </c>
-      <c r="CE1" t="inlineStr">
+      <c r="CE1" s="1" t="inlineStr">
         <is>
           <t>Marathon Oil Corporation</t>
         </is>
       </c>
-      <c r="CF1" t="inlineStr">
+      <c r="CF1" s="1" t="inlineStr">
         <is>
           <t>MEDNAX, Inc.</t>
         </is>
       </c>
-      <c r="CG1" t="inlineStr">
+      <c r="CG1" s="1" t="inlineStr">
         <is>
           <t>Meridian Bancorp Inc</t>
         </is>
       </c>
-      <c r="CH1" t="inlineStr">
+      <c r="CH1" s="1" t="inlineStr">
         <is>
           <t>Monro Inc</t>
         </is>
       </c>
-      <c r="CI1" t="inlineStr">
+      <c r="CI1" s="1" t="inlineStr">
         <is>
           <t>Murphy Oil Corporation</t>
         </is>
       </c>
-      <c r="CJ1" t="inlineStr">
+      <c r="CJ1" s="1" t="inlineStr">
         <is>
           <t>NOV Inc.</t>
         </is>
       </c>
-      <c r="CK1" t="inlineStr">
+      <c r="CK1" s="1" t="inlineStr">
         <is>
           <t>Natus Medical Incorporated</t>
         </is>
       </c>
-      <c r="CL1" t="inlineStr">
+      <c r="CL1" s="1" t="inlineStr">
         <is>
           <t>Neenah Inc</t>
         </is>
       </c>
-      <c r="CM1" t="inlineStr">
+      <c r="CM1" s="1" t="inlineStr">
         <is>
           <t>New Residential Investment Corp.</t>
         </is>
       </c>
-      <c r="CN1" t="inlineStr">
+      <c r="CN1" s="1" t="inlineStr">
         <is>
           <t>NMI Holdings, Inc. Class A</t>
         </is>
       </c>
-      <c r="CO1" t="inlineStr">
+      <c r="CO1" s="1" t="inlineStr">
         <is>
           <t>Nordstrom, Inc.</t>
         </is>
       </c>
-      <c r="CP1" t="inlineStr">
+      <c r="CP1" s="1" t="inlineStr">
         <is>
           <t>Northwest Natural Holding Co.</t>
         </is>
       </c>
-      <c r="CQ1" t="inlineStr">
+      <c r="CQ1" s="1" t="inlineStr">
         <is>
           <t>Norwegian Cruise Line Holdings Ltd.</t>
         </is>
       </c>
-      <c r="CR1" t="inlineStr">
+      <c r="CR1" s="1" t="inlineStr">
         <is>
           <t>NuVasive, Inc.</t>
         </is>
       </c>
-      <c r="CS1" t="inlineStr">
+      <c r="CS1" s="1" t="inlineStr">
         <is>
           <t>Occidental Petroleum Corporation</t>
         </is>
       </c>
-      <c r="CT1" t="inlineStr">
+      <c r="CT1" s="1" t="inlineStr">
         <is>
           <t>OceanFirst Financial Corp.</t>
         </is>
       </c>
-      <c r="CU1" t="inlineStr">
+      <c r="CU1" s="1" t="inlineStr">
         <is>
           <t>ONEOK, Inc.</t>
         </is>
       </c>
-      <c r="CV1" t="inlineStr">
+      <c r="CV1" s="1" t="inlineStr">
         <is>
           <t>OUTFRONT Media Inc.</t>
         </is>
       </c>
-      <c r="CW1" t="inlineStr">
+      <c r="CW1" s="1" t="inlineStr">
         <is>
           <t>PacWest Bancorp</t>
         </is>
       </c>
-      <c r="CX1" t="inlineStr">
+      <c r="CX1" s="1" t="inlineStr">
         <is>
           <t>Pebblebrook Hotel Trust</t>
         </is>
       </c>
-      <c r="CY1" t="inlineStr">
+      <c r="CY1" s="1" t="inlineStr">
         <is>
           <t>Phillips 66</t>
         </is>
       </c>
-      <c r="CZ1" t="inlineStr">
+      <c r="CZ1" s="1" t="inlineStr">
         <is>
           <t>Photronics, Inc.</t>
         </is>
       </c>
-      <c r="DA1" t="inlineStr">
+      <c r="DA1" s="1" t="inlineStr">
         <is>
           <t>Pilgrims Pride Corporation</t>
         </is>
       </c>
-      <c r="DB1" t="inlineStr">
+      <c r="DB1" s="1" t="inlineStr">
         <is>
           <t>ProAssurance Corporation</t>
         </is>
       </c>
-      <c r="DC1" t="inlineStr">
+      <c r="DC1" s="1" t="inlineStr">
         <is>
           <t>PROS Holdings, Inc.</t>
         </is>
       </c>
-      <c r="DD1" t="inlineStr">
+      <c r="DD1" s="1" t="inlineStr">
         <is>
           <t>Provident Financial Services, Inc.</t>
         </is>
       </c>
-      <c r="DE1" t="inlineStr">
+      <c r="DE1" s="1" t="inlineStr">
         <is>
           <t>Retail Properties of America, Inc. Class A</t>
         </is>
       </c>
-      <c r="DF1" t="inlineStr">
+      <c r="DF1" s="1" t="inlineStr">
         <is>
           <t>Rite Aid Corporation</t>
         </is>
       </c>
-      <c r="DG1" t="inlineStr">
+      <c r="DG1" s="1" t="inlineStr">
         <is>
           <t>RLJ Lodging Trust</t>
         </is>
       </c>
-      <c r="DH1" t="inlineStr">
+      <c r="DH1" s="1" t="inlineStr">
         <is>
           <t>Royal Caribbean Group</t>
         </is>
       </c>
-      <c r="DI1" t="inlineStr">
+      <c r="DI1" s="1" t="inlineStr">
         <is>
           <t>Ryman Hospitality Properties, Inc.</t>
         </is>
       </c>
-      <c r="DJ1" t="inlineStr">
+      <c r="DJ1" s="1" t="inlineStr">
         <is>
           <t>S&amp;T Bancorp, Inc.</t>
         </is>
       </c>
-      <c r="DK1" t="inlineStr">
+      <c r="DK1" s="1" t="inlineStr">
         <is>
           <t>Sabre Corp.</t>
         </is>
       </c>
-      <c r="DL1" t="inlineStr">
+      <c r="DL1" s="1" t="inlineStr">
         <is>
           <t>Sally Beauty Holdings, Inc.</t>
         </is>
       </c>
-      <c r="DM1" t="inlineStr">
+      <c r="DM1" s="1" t="inlineStr">
         <is>
           <t>Saul Centers, Inc.</t>
         </is>
       </c>
-      <c r="DN1" t="inlineStr">
+      <c r="DN1" s="1" t="inlineStr">
         <is>
           <t>Schlumberger NV</t>
         </is>
       </c>
-      <c r="DO1" t="inlineStr">
+      <c r="DO1" s="1" t="inlineStr">
         <is>
           <t>Scholastic Corporation</t>
         </is>
       </c>
-      <c r="DP1" t="inlineStr">
+      <c r="DP1" s="1" t="inlineStr">
         <is>
           <t>SFL Corporation Limited</t>
         </is>
       </c>
-      <c r="DQ1" t="inlineStr">
+      <c r="DQ1" s="1" t="inlineStr">
         <is>
           <t>Simon Property Group, Inc.</t>
         </is>
       </c>
-      <c r="DR1" t="inlineStr">
+      <c r="DR1" s="1" t="inlineStr">
         <is>
           <t>Six Flags Entertainment Corporation</t>
         </is>
       </c>
-      <c r="DS1" t="inlineStr">
+      <c r="DS1" s="1" t="inlineStr">
         <is>
           <t>SkyWest, Inc</t>
         </is>
       </c>
-      <c r="DT1" t="inlineStr">
+      <c r="DT1" s="1" t="inlineStr">
         <is>
           <t>SL Green Realty Corp.</t>
         </is>
       </c>
-      <c r="DU1" t="inlineStr">
+      <c r="DU1" s="1" t="inlineStr">
         <is>
           <t>Spirit AeroSystems Holdings, Inc. Class A</t>
         </is>
       </c>
-      <c r="DV1" t="inlineStr">
+      <c r="DV1" s="1" t="inlineStr">
         <is>
           <t>Spirit Airlines, Inc.</t>
         </is>
       </c>
-      <c r="DW1" t="inlineStr">
+      <c r="DW1" s="1" t="inlineStr">
         <is>
           <t>Steelcase Inc. Class A</t>
         </is>
       </c>
-      <c r="DX1" t="inlineStr">
+      <c r="DX1" s="1" t="inlineStr">
         <is>
           <t>Strategic Education, Inc.</t>
         </is>
       </c>
-      <c r="DY1" t="inlineStr">
+      <c r="DY1" s="1" t="inlineStr">
         <is>
           <t>Targa Resources Corp.</t>
         </is>
       </c>
-      <c r="DZ1" t="inlineStr">
+      <c r="DZ1" s="1" t="inlineStr">
         <is>
           <t>Theravance Biopharma Inc</t>
         </is>
       </c>
-      <c r="EA1" t="inlineStr">
+      <c r="EA1" s="1" t="inlineStr">
         <is>
           <t>Two Harbors Investment Corp.</t>
         </is>
       </c>
-      <c r="EB1" t="inlineStr">
+      <c r="EB1" s="1" t="inlineStr">
         <is>
           <t>United Airlines Holdings, Inc.</t>
         </is>
       </c>
-      <c r="EC1" t="inlineStr">
+      <c r="EC1" s="1" t="inlineStr">
         <is>
           <t>Universal Health Realty Income Trust</t>
         </is>
       </c>
-      <c r="ED1" t="inlineStr">
+      <c r="ED1" s="1" t="inlineStr">
         <is>
           <t>US Ecology, Inc.</t>
         </is>
       </c>
-      <c r="EE1" t="inlineStr">
+      <c r="EE1" s="1" t="inlineStr">
         <is>
           <t>Valero Energy Corporation</t>
         </is>
       </c>
-      <c r="EF1" t="inlineStr">
+      <c r="EF1" s="1" t="inlineStr">
         <is>
           <t>ViaSat, Inc.</t>
         </is>
       </c>
-      <c r="EG1" t="inlineStr">
+      <c r="EG1" s="1" t="inlineStr">
         <is>
           <t>Vornado Realty Trust</t>
         </is>
       </c>
-      <c r="EH1" t="inlineStr">
+      <c r="EH1" s="1" t="inlineStr">
         <is>
           <t>Walgreens Boots Alliance Inc</t>
         </is>
       </c>
-      <c r="EI1" t="inlineStr">
+      <c r="EI1" s="1" t="inlineStr">
         <is>
           <t>Washington Federal, Inc.</t>
         </is>
       </c>
-      <c r="EJ1" t="inlineStr">
+      <c r="EJ1" s="1" t="inlineStr">
         <is>
           <t>Wells Fargo &amp; Company</t>
         </is>
       </c>
-      <c r="EK1" t="inlineStr">
+      <c r="EK1" s="1" t="inlineStr">
         <is>
           <t>World Fuel Services Corporation</t>
         </is>
       </c>
-      <c r="EL1" t="inlineStr">
+      <c r="EL1" s="1" t="inlineStr">
         <is>
           <t>World Wrestling Entertainment, Inc. Class A</t>
         </is>
       </c>
-      <c r="EM1" t="inlineStr">
+      <c r="EM1" s="1" t="inlineStr">
         <is>
           <t>WPX Energy, Inc.</t>
         </is>
       </c>
-      <c r="EN1" t="inlineStr">
+      <c r="EN1" s="1" t="inlineStr">
         <is>
           <t>Wynn Resorts, Limited</t>
         </is>
       </c>
-      <c r="EO1" t="inlineStr">
+      <c r="EO1" s="1" t="inlineStr">
         <is>
           <t>Xerox Holdings Corporation</t>
         </is>
       </c>
-      <c r="EP1" t="inlineStr">
+      <c r="EP1" s="1" t="inlineStr">
         <is>
           <t>Zogenix, Inc.</t>
         </is>
       </c>
-      <c r="EQ1" t="inlineStr">
+      <c r="EQ1" s="1" t="inlineStr">
         <is>
           <t>Xenia Hotels &amp; Resorts, Inc.</t>
         </is>
       </c>
-      <c r="ER1" t="inlineStr">
+      <c r="ER1" s="1" t="inlineStr">
         <is>
           <t>Paramount Group, Inc.</t>
         </is>
       </c>
-      <c r="ES1" t="inlineStr">
+      <c r="ES1" s="1" t="inlineStr">
         <is>
           <t>Urban Edge Properties</t>
         </is>
       </c>
-      <c r="ET1" t="inlineStr">
+      <c r="ET1" s="1" t="inlineStr">
         <is>
           <t>Esperion Therapeutics, Inc.</t>
         </is>
       </c>
-      <c r="EU1" t="inlineStr">
+      <c r="EU1" s="1" t="inlineStr">
         <is>
           <t>uniQure N.V.</t>
         </is>
       </c>
-      <c r="EV1" t="inlineStr">
+      <c r="EV1" s="1" t="inlineStr">
         <is>
           <t>Great Western Bancorp, Inc.</t>
         </is>
       </c>
-      <c r="EW1" t="inlineStr">
+      <c r="EW1" s="1" t="inlineStr">
         <is>
           <t>Global Blood Therapeutics Inc</t>
         </is>
       </c>
-      <c r="EX1" t="inlineStr">
+      <c r="EX1" s="1" t="inlineStr">
         <is>
           <t>Hewlett Packard Enterprise Co.</t>
         </is>
       </c>
-      <c r="EY1" t="inlineStr">
+      <c r="EY1" s="1" t="inlineStr">
         <is>
           <t>Welbilt Inc</t>
         </is>
       </c>
-      <c r="EZ1" t="inlineStr">
+      <c r="EZ1" s="1" t="inlineStr">
         <is>
           <t>Park Hotels &amp; Resorts, Inc.</t>
         </is>
       </c>
-      <c r="FA1" t="inlineStr">
+      <c r="FA1" s="1" t="inlineStr">
         <is>
           <t>TechnipFMC Plc</t>
         </is>
       </c>
-      <c r="FB1" t="inlineStr">
+      <c r="FB1" s="1" t="inlineStr">
         <is>
           <t>Tactile Systems Technology, Inc.</t>
         </is>
       </c>
-      <c r="FC1" t="inlineStr">
+      <c r="FC1" s="1" t="inlineStr">
         <is>
           <t>Bausch Health Companies Inc.</t>
         </is>
       </c>
-      <c r="FD1" t="inlineStr">
+      <c r="FD1" s="1" t="inlineStr">
         <is>
           <t>Frontline Ltd.</t>
         </is>
       </c>
-      <c r="FE1" t="inlineStr">
+      <c r="FE1" s="1" t="inlineStr">
         <is>
           <t>Plains GP Holdings LP Class A</t>
         </is>
       </c>
-      <c r="FF1" t="inlineStr">
+      <c r="FF1" s="1" t="inlineStr">
         <is>
           <t>Liberty Latin America Ltd. Class C</t>
         </is>
       </c>
-      <c r="FG1" t="inlineStr">
+      <c r="FG1" s="1" t="inlineStr">
         <is>
           <t>Scorpio Tankers Inc.</t>
         </is>
       </c>
-      <c r="FH1" t="inlineStr">
+      <c r="FH1" s="1" t="inlineStr">
         <is>
           <t>Tabula Rasa Healthcare, Inc.</t>
         </is>
       </c>
-      <c r="FI1" t="inlineStr">
+      <c r="FI1" s="1" t="inlineStr">
         <is>
           <t>GrafTech International Ltd.</t>
         </is>
       </c>
-      <c r="FJ1" t="inlineStr">
+      <c r="FJ1" s="1" t="inlineStr">
         <is>
           <t>Equitrans Midstream Corp.</t>
         </is>
       </c>
-      <c r="FK1" t="inlineStr">
+      <c r="FK1" s="1" t="inlineStr">
         <is>
           <t>Axsome Therapeutics, Inc.</t>
         </is>
       </c>
-      <c r="FL1" t="inlineStr">
+      <c r="FL1" s="1" t="inlineStr">
         <is>
           <t>Arvinas, Inc.</t>
         </is>
       </c>
-      <c r="FM1" t="inlineStr">
+      <c r="FM1" s="1" t="inlineStr">
         <is>
           <t>Coronado Global Resources Inc. Shs Chess Depository Interests Repr 10 Sh</t>
         </is>
       </c>
-      <c r="FN1" t="inlineStr">
+      <c r="FN1" s="1" t="inlineStr">
         <is>
           <t>Gossamer Bio, Inc.</t>
         </is>
       </c>
-      <c r="FO1" t="inlineStr">
+      <c r="FO1" s="1" t="inlineStr">
         <is>
           <t>CarGurus, Inc. Class A</t>
         </is>
       </c>
-      <c r="FP1" t="inlineStr">
+      <c r="FP1" s="1" t="inlineStr">
         <is>
           <t>Ovintiv Inc</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>2020-01-03</t>
         </is>
@@ -2083,7 +2095,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>2020-01-10</t>
         </is>
@@ -2603,7 +2615,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>2020-01-17</t>
         </is>
@@ -3123,7 +3135,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>2020-01-24</t>
         </is>
@@ -3643,7 +3655,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>2020-01-31</t>
         </is>
@@ -4163,7 +4175,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>2020-02-07</t>
         </is>
@@ -4683,7 +4695,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>2020-02-14</t>
         </is>
@@ -5203,7 +5215,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>2020-02-21</t>
         </is>
@@ -5723,7 +5735,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>2020-02-28</t>
         </is>
@@ -6243,7 +6255,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>2020-03-06</t>
         </is>
@@ -6763,7 +6775,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>2020-03-13</t>
         </is>
@@ -7283,7 +7295,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>2020-03-20</t>
         </is>
@@ -7803,7 +7815,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>2020-03-27</t>
         </is>
@@ -8323,7 +8335,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>2020-04-03</t>
         </is>
@@ -8843,7 +8855,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>2020-04-10</t>
         </is>
@@ -9363,7 +9375,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>2020-04-17</t>
         </is>
@@ -9883,7 +9895,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>2020-04-24</t>
         </is>
@@ -10403,7 +10415,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>2020-05-01</t>
         </is>
@@ -10923,7 +10935,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>2020-05-08</t>
         </is>
@@ -11443,7 +11455,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>2020-05-15</t>
         </is>
@@ -11963,7 +11975,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>2020-05-22</t>
         </is>
@@ -12483,7 +12495,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>2020-05-29</t>
         </is>
@@ -13003,7 +13015,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>2020-06-05</t>
         </is>
@@ -13523,7 +13535,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>2020-06-12</t>
         </is>
@@ -14043,7 +14055,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>2020-06-19</t>
         </is>
@@ -14563,7 +14575,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>2020-06-26</t>
         </is>
@@ -15083,7 +15095,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>2020-07-03</t>
         </is>
@@ -15603,7 +15615,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>2020-07-10</t>
         </is>
@@ -16123,7 +16135,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="1" t="inlineStr">
         <is>
           <t>2020-07-17</t>
         </is>
@@ -16643,7 +16655,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>2020-07-24</t>
         </is>
@@ -17163,7 +17175,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>2020-07-31</t>
         </is>
@@ -17683,7 +17695,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="1" t="inlineStr">
         <is>
           <t>2020-08-07</t>
         </is>
@@ -18203,7 +18215,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="1" t="inlineStr">
         <is>
           <t>2020-08-14</t>
         </is>
@@ -18723,7 +18735,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="1" t="inlineStr">
         <is>
           <t>2020-08-21</t>
         </is>
@@ -19243,7 +19255,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="1" t="inlineStr">
         <is>
           <t>2020-08-28</t>
         </is>
@@ -19763,7 +19775,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="1" t="inlineStr">
         <is>
           <t>2020-09-04</t>
         </is>
@@ -20283,7 +20295,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="1" t="inlineStr">
         <is>
           <t>2020-09-11</t>
         </is>
@@ -20803,7 +20815,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="1" t="inlineStr">
         <is>
           <t>2020-09-18</t>
         </is>
@@ -21323,7 +21335,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="1" t="inlineStr">
         <is>
           <t>2020-09-25</t>
         </is>
@@ -21843,7 +21855,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="1" t="inlineStr">
         <is>
           <t>2020-10-02</t>
         </is>
@@ -22363,7 +22375,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="1" t="inlineStr">
         <is>
           <t>2020-10-09</t>
         </is>
@@ -22883,7 +22895,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="1" t="inlineStr">
         <is>
           <t>2020-10-16</t>
         </is>
@@ -23403,7 +23415,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="1" t="inlineStr">
         <is>
           <t>2020-10-23</t>
         </is>
@@ -23923,7 +23935,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="1" t="inlineStr">
         <is>
           <t>2020-10-30</t>
         </is>
@@ -24443,7 +24455,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="1" t="inlineStr">
         <is>
           <t>2020-11-06</t>
         </is>
@@ -24963,7 +24975,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="1" t="inlineStr">
         <is>
           <t>2020-11-13</t>
         </is>
@@ -25483,7 +25495,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="1" t="inlineStr">
         <is>
           <t>2020-11-20</t>
         </is>
@@ -26003,7 +26015,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="1" t="inlineStr">
         <is>
           <t>2020-11-27</t>
         </is>
@@ -26523,7 +26535,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="1" t="inlineStr">
         <is>
           <t>2020-12-04</t>
         </is>
@@ -27043,7 +27055,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="1" t="inlineStr">
         <is>
           <t>2020-12-11</t>
         </is>
@@ -27563,7 +27575,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="1" t="inlineStr">
         <is>
           <t>2020-12-18</t>
         </is>
@@ -28083,7 +28095,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="1" t="inlineStr">
         <is>
           <t>2020-12-25</t>
         </is>
@@ -28617,869 +28629,869 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Acceleron Pharma Inc</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Advanced Drainage Systems, Inc.</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Advanced Micro Devices, Inc.</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Albemarle Corporation</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Align Technology, Inc.</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Altra Industrial Motion Corp.</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Amazon.com, Inc.</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Amicus Therapeutics, Inc.</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Boston Beer Company, Inc. Class A</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Brooks Automation, Inc.</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Cadence Design Systems, Inc.</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Canadian Solar Inc.</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Chegg, Inc.</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Corcept Therapeutics Incorporated.</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Cree, Inc.</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Cytokinetics, Incorporated</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Darling Ingredients Inc.</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Enphase Energy, Inc.</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Entegris, Inc.</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>FedEx Corporation</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>First Solar, Inc.</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Freeport-McMoRan, Inc.</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Freshpet Inc</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Generac Holdings Inc.</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Glu Mobile Inc.</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Green Dot Corporation Class A</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Halozyme Therapeutics, Inc.</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Hannon Armstrong Sustainable Infrastructure Capital, Inc.</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Horizon Therapeutics Public Limited Company</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>HubSpot, Inc.</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>IDEXX Laboratories, Inc.</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>II-VI Incorporated</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Inphi Corporation</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>L Brands, Inc.</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Lattice Semiconductor Corporation</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Qurate Retail, Inc. Class A</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Lithia Motors, Inc. Class A</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Marvell Technology Group Ltd.</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Medifast, Inc.</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>Merit Medical Systems, Inc.</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>MicroStrategy Incorporated Class A</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>Monolithic Power Systems, Inc.</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>NanoString Technologies, Inc.</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>Nuance Communications, Inc.</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>NVIDIA Corporation</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>Paylocity Holding Corp.</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>Pegasystems Inc.</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>Penn National Gaming, Inc.</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>PennyMac Financial Services, Inc.</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>Plug Power Inc.</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>ModivCare Inc.</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>Qualcomm Inc</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BB1" s="1" t="inlineStr">
         <is>
           <t>Quanta Services, Inc.</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BC1" s="1" t="inlineStr">
         <is>
           <t>Quidel Corporation</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BD1" s="1" t="inlineStr">
         <is>
           <t>Range Resources Corporation</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>Renewable Energy Group, Inc.</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>Repligen Corporation</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BG1" s="1" t="inlineStr">
         <is>
           <t>RH</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BH1" s="1" t="inlineStr">
         <is>
           <t>RingCentral, Inc. Class A</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BI1" s="1" t="inlineStr">
         <is>
           <t>Rollins, Inc.</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BJ1" s="1" t="inlineStr">
         <is>
           <t>Saia, Inc.</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BK1" s="1" t="inlineStr">
         <is>
           <t>Scotts Miracle-Gro Company Class A</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BL1" s="1" t="inlineStr">
         <is>
           <t>ServiceNow, Inc.</t>
         </is>
       </c>
-      <c r="BM1" t="inlineStr">
+      <c r="BM1" s="1" t="inlineStr">
         <is>
           <t>SPS Commerce, Inc.</t>
         </is>
       </c>
-      <c r="BN1" t="inlineStr">
+      <c r="BN1" s="1" t="inlineStr">
         <is>
           <t>St. Joe Company</t>
         </is>
       </c>
-      <c r="BO1" t="inlineStr">
+      <c r="BO1" s="1" t="inlineStr">
         <is>
           <t>STAAR Surgical Company</t>
         </is>
       </c>
-      <c r="BP1" t="inlineStr">
+      <c r="BP1" s="1" t="inlineStr">
         <is>
           <t>Stamps.com Inc.</t>
         </is>
       </c>
-      <c r="BQ1" t="inlineStr">
+      <c r="BQ1" s="1" t="inlineStr">
         <is>
           <t>BMC Stock Holdings, Inc.</t>
         </is>
       </c>
-      <c r="BR1" t="inlineStr">
+      <c r="BR1" s="1" t="inlineStr">
         <is>
           <t>SunPower Corporation</t>
         </is>
       </c>
-      <c r="BS1" t="inlineStr">
+      <c r="BS1" s="1" t="inlineStr">
         <is>
           <t>T-Mobile US, Inc.</t>
         </is>
       </c>
-      <c r="BT1" t="inlineStr">
+      <c r="BT1" s="1" t="inlineStr">
         <is>
           <t>Axon Enterprise Inc</t>
         </is>
       </c>
-      <c r="BU1" t="inlineStr">
+      <c r="BU1" s="1" t="inlineStr">
         <is>
           <t>TechTarget, Inc.</t>
         </is>
       </c>
-      <c r="BV1" t="inlineStr">
+      <c r="BV1" s="1" t="inlineStr">
         <is>
           <t>TTEC Holdings, Inc.</t>
         </is>
       </c>
-      <c r="BW1" t="inlineStr">
+      <c r="BW1" s="1" t="inlineStr">
         <is>
           <t>Tesla Inc</t>
         </is>
       </c>
-      <c r="BX1" t="inlineStr">
+      <c r="BX1" s="1" t="inlineStr">
         <is>
           <t>TG Therapeutics, Inc.</t>
         </is>
       </c>
-      <c r="BY1" t="inlineStr">
+      <c r="BY1" s="1" t="inlineStr">
         <is>
           <t>Trex Company, Inc.</t>
         </is>
       </c>
-      <c r="BZ1" t="inlineStr">
+      <c r="BZ1" s="1" t="inlineStr">
         <is>
           <t>Ultragenyx Pharmaceutical, Inc.</t>
         </is>
       </c>
-      <c r="CA1" t="inlineStr">
+      <c r="CA1" s="1" t="inlineStr">
         <is>
           <t>Veeva Systems Inc Class A</t>
         </is>
       </c>
-      <c r="CB1" t="inlineStr">
+      <c r="CB1" s="1" t="inlineStr">
         <is>
           <t>Veracyte Inc</t>
         </is>
       </c>
-      <c r="CC1" t="inlineStr">
+      <c r="CC1" s="1" t="inlineStr">
         <is>
           <t>Vicor Corporation</t>
         </is>
       </c>
-      <c r="CD1" t="inlineStr">
+      <c r="CD1" s="1" t="inlineStr">
         <is>
           <t>Vonage Holdings Corp.</t>
         </is>
       </c>
-      <c r="CE1" t="inlineStr">
+      <c r="CE1" s="1" t="inlineStr">
         <is>
           <t>Wayfair, Inc. Class A</t>
         </is>
       </c>
-      <c r="CF1" t="inlineStr">
+      <c r="CF1" s="1" t="inlineStr">
         <is>
           <t>West Pharmaceutical Services, Inc.</t>
         </is>
       </c>
-      <c r="CG1" t="inlineStr">
+      <c r="CG1" s="1" t="inlineStr">
         <is>
           <t>Wix.com Ltd.</t>
         </is>
       </c>
-      <c r="CH1" t="inlineStr">
+      <c r="CH1" s="1" t="inlineStr">
         <is>
           <t>Zendesk, Inc.</t>
         </is>
       </c>
-      <c r="CI1" t="inlineStr">
+      <c r="CI1" s="1" t="inlineStr">
         <is>
           <t>Zillow Group, Inc. Class A</t>
         </is>
       </c>
-      <c r="CJ1" t="inlineStr">
+      <c r="CJ1" s="1" t="inlineStr">
         <is>
           <t>Invitae Corp.</t>
         </is>
       </c>
-      <c r="CK1" t="inlineStr">
+      <c r="CK1" s="1" t="inlineStr">
         <is>
           <t>Etsy, Inc.</t>
         </is>
       </c>
-      <c r="CL1" t="inlineStr">
+      <c r="CL1" s="1" t="inlineStr">
         <is>
           <t>TopBuild Corp.</t>
         </is>
       </c>
-      <c r="CM1" t="inlineStr">
+      <c r="CM1" s="1" t="inlineStr">
         <is>
           <t>SolarEdge Technologies, Inc.</t>
         </is>
       </c>
-      <c r="CN1" t="inlineStr">
+      <c r="CN1" s="1" t="inlineStr">
         <is>
           <t>Kornit Digital Ltd.</t>
         </is>
       </c>
-      <c r="CO1" t="inlineStr">
+      <c r="CO1" s="1" t="inlineStr">
         <is>
           <t>PayPal Holdings Inc</t>
         </is>
       </c>
-      <c r="CP1" t="inlineStr">
+      <c r="CP1" s="1" t="inlineStr">
         <is>
           <t>Zillow Group, Inc. Class C</t>
         </is>
       </c>
-      <c r="CQ1" t="inlineStr">
+      <c r="CQ1" s="1" t="inlineStr">
         <is>
           <t>Workiva, Inc. Class A</t>
         </is>
       </c>
-      <c r="CR1" t="inlineStr">
+      <c r="CR1" s="1" t="inlineStr">
         <is>
           <t>Fate Therapeutics, Inc.</t>
         </is>
       </c>
-      <c r="CS1" t="inlineStr">
+      <c r="CS1" s="1" t="inlineStr">
         <is>
           <t>Catalent Inc</t>
         </is>
       </c>
-      <c r="CT1" t="inlineStr">
+      <c r="CT1" s="1" t="inlineStr">
         <is>
           <t>Mirati Therapeutics Inc.</t>
         </is>
       </c>
-      <c r="CU1" t="inlineStr">
+      <c r="CU1" s="1" t="inlineStr">
         <is>
           <t>Sunrun Inc.</t>
         </is>
       </c>
-      <c r="CV1" t="inlineStr">
+      <c r="CV1" s="1" t="inlineStr">
         <is>
           <t>Five9, Inc.</t>
         </is>
       </c>
-      <c r="CW1" t="inlineStr">
+      <c r="CW1" s="1" t="inlineStr">
         <is>
           <t>Teladoc Health, Inc.</t>
         </is>
       </c>
-      <c r="CX1" t="inlineStr">
+      <c r="CX1" s="1" t="inlineStr">
         <is>
           <t>Alarm.com Holdings, Inc.</t>
         </is>
       </c>
-      <c r="CY1" t="inlineStr">
+      <c r="CY1" s="1" t="inlineStr">
         <is>
           <t>Natera, Inc.</t>
         </is>
       </c>
-      <c r="CZ1" t="inlineStr">
+      <c r="CZ1" s="1" t="inlineStr">
         <is>
           <t>Trupanion, Inc.</t>
         </is>
       </c>
-      <c r="DA1" t="inlineStr">
+      <c r="DA1" s="1" t="inlineStr">
         <is>
           <t>Square, Inc. Class A</t>
         </is>
       </c>
-      <c r="DB1" t="inlineStr">
+      <c r="DB1" s="1" t="inlineStr">
         <is>
           <t>Intellia Therapeutics, Inc.</t>
         </is>
       </c>
-      <c r="DC1" t="inlineStr">
+      <c r="DC1" s="1" t="inlineStr">
         <is>
           <t>Atlassian Corp. Plc Class A</t>
         </is>
       </c>
-      <c r="DD1" t="inlineStr">
+      <c r="DD1" s="1" t="inlineStr">
         <is>
           <t>Kinsale Capital Group, Inc.</t>
         </is>
       </c>
-      <c r="DE1" t="inlineStr">
+      <c r="DE1" s="1" t="inlineStr">
         <is>
           <t>Twilio, Inc. Class A</t>
         </is>
       </c>
-      <c r="DF1" t="inlineStr">
+      <c r="DF1" s="1" t="inlineStr">
         <is>
           <t>Coupa Software, Inc.</t>
         </is>
       </c>
-      <c r="DG1" t="inlineStr">
+      <c r="DG1" s="1" t="inlineStr">
         <is>
           <t>iRhythm Technologies, Inc.</t>
         </is>
       </c>
-      <c r="DH1" t="inlineStr">
+      <c r="DH1" s="1" t="inlineStr">
         <is>
           <t>Trade Desk, Inc. Class A</t>
         </is>
       </c>
-      <c r="DI1" t="inlineStr">
+      <c r="DI1" s="1" t="inlineStr">
         <is>
           <t>BlackLine, Inc.</t>
         </is>
       </c>
-      <c r="DJ1" t="inlineStr">
+      <c r="DJ1" s="1" t="inlineStr">
         <is>
           <t>Safehold Inc.</t>
         </is>
       </c>
-      <c r="DK1" t="inlineStr">
+      <c r="DK1" s="1" t="inlineStr">
         <is>
           <t>Okta, Inc. Class A</t>
         </is>
       </c>
-      <c r="DL1" t="inlineStr">
+      <c r="DL1" s="1" t="inlineStr">
         <is>
           <t>Apellis Pharmaceuticals, Inc.</t>
         </is>
       </c>
-      <c r="DM1" t="inlineStr">
+      <c r="DM1" s="1" t="inlineStr">
         <is>
           <t>Simulations Plus, Inc.</t>
         </is>
       </c>
-      <c r="DN1" t="inlineStr">
+      <c r="DN1" s="1" t="inlineStr">
         <is>
           <t>Shopify, Inc. Class A</t>
         </is>
       </c>
-      <c r="DO1" t="inlineStr">
+      <c r="DO1" s="1" t="inlineStr">
         <is>
           <t>Carvana Co. Class A</t>
         </is>
       </c>
-      <c r="DP1" t="inlineStr">
+      <c r="DP1" s="1" t="inlineStr">
         <is>
           <t>MercadoLibre, Inc.</t>
         </is>
       </c>
-      <c r="DQ1" t="inlineStr">
+      <c r="DQ1" s="1" t="inlineStr">
         <is>
           <t>Redfin Corporation</t>
         </is>
       </c>
-      <c r="DR1" t="inlineStr">
+      <c r="DR1" s="1" t="inlineStr">
         <is>
           <t>Denali Therapeutics Inc.</t>
         </is>
       </c>
-      <c r="DS1" t="inlineStr">
+      <c r="DS1" s="1" t="inlineStr">
         <is>
           <t>SailPoint Technologies Holdings, Inc.</t>
         </is>
       </c>
-      <c r="DT1" t="inlineStr">
+      <c r="DT1" s="1" t="inlineStr">
         <is>
           <t>CRISPR Therapeutics AG</t>
         </is>
       </c>
-      <c r="DU1" t="inlineStr">
+      <c r="DU1" s="1" t="inlineStr">
         <is>
           <t>Inspire Medical Systems, Inc.</t>
         </is>
       </c>
-      <c r="DV1" t="inlineStr">
+      <c r="DV1" s="1" t="inlineStr">
         <is>
           <t>CareDx, Inc.</t>
         </is>
       </c>
-      <c r="DW1" t="inlineStr">
+      <c r="DW1" s="1" t="inlineStr">
         <is>
           <t>Zscaler, Inc.</t>
         </is>
       </c>
-      <c r="DX1" t="inlineStr">
+      <c r="DX1" s="1" t="inlineStr">
         <is>
           <t>BJs Wholesale Club Holdings, Inc.</t>
         </is>
       </c>
-      <c r="DY1" t="inlineStr">
+      <c r="DY1" s="1" t="inlineStr">
         <is>
           <t>Snap, Inc. Class A</t>
         </is>
       </c>
-      <c r="DZ1" t="inlineStr">
+      <c r="DZ1" s="1" t="inlineStr">
         <is>
           <t>Spotify Technology SA</t>
         </is>
       </c>
-      <c r="EA1" t="inlineStr">
+      <c r="EA1" s="1" t="inlineStr">
         <is>
           <t>Covetrus, Inc.</t>
         </is>
       </c>
-      <c r="EB1" t="inlineStr">
+      <c r="EB1" s="1" t="inlineStr">
         <is>
           <t>Nova Measuring Instruments Ltd</t>
         </is>
       </c>
-      <c r="EC1" t="inlineStr">
+      <c r="EC1" s="1" t="inlineStr">
         <is>
           <t>YETI Holdings, Inc.</t>
         </is>
       </c>
-      <c r="ED1" t="inlineStr">
+      <c r="ED1" s="1" t="inlineStr">
         <is>
           <t>MongoDB, Inc. Class A</t>
         </is>
       </c>
-      <c r="EE1" t="inlineStr">
+      <c r="EE1" s="1" t="inlineStr">
         <is>
           <t>Avalara Inc</t>
         </is>
       </c>
-      <c r="EF1" t="inlineStr">
+      <c r="EF1" s="1" t="inlineStr">
         <is>
           <t>Twist Bioscience Corp.</t>
         </is>
       </c>
-      <c r="EG1" t="inlineStr">
+      <c r="EG1" s="1" t="inlineStr">
         <is>
           <t>CryoPort, Inc.</t>
         </is>
       </c>
-      <c r="EH1" t="inlineStr">
+      <c r="EH1" s="1" t="inlineStr">
         <is>
           <t>Repay Holdings Corp. Class A</t>
         </is>
       </c>
-      <c r="EI1" t="inlineStr">
+      <c r="EI1" s="1" t="inlineStr">
         <is>
           <t>Roku, Inc. Class A</t>
         </is>
       </c>
-      <c r="EJ1" t="inlineStr">
+      <c r="EJ1" s="1" t="inlineStr">
         <is>
           <t>Appian Corporation Class A</t>
         </is>
       </c>
-      <c r="EK1" t="inlineStr">
+      <c r="EK1" s="1" t="inlineStr">
         <is>
           <t>Innovative Industrial Properties Inc</t>
         </is>
       </c>
-      <c r="EL1" t="inlineStr">
+      <c r="EL1" s="1" t="inlineStr">
         <is>
           <t>Farfetch Limited Class A</t>
         </is>
       </c>
-      <c r="EM1" t="inlineStr">
+      <c r="EM1" s="1" t="inlineStr">
         <is>
           <t>Goosehead Insurance, Inc. Class A</t>
         </is>
       </c>
-      <c r="EN1" t="inlineStr">
+      <c r="EN1" s="1" t="inlineStr">
         <is>
           <t>Virgin Galactic Holdings Inc</t>
         </is>
       </c>
-      <c r="EO1" t="inlineStr">
+      <c r="EO1" s="1" t="inlineStr">
         <is>
           <t>Upwork, Inc.</t>
         </is>
       </c>
-      <c r="EP1" t="inlineStr">
+      <c r="EP1" s="1" t="inlineStr">
         <is>
           <t>Shockwave Medical, Inc.</t>
         </is>
       </c>
-      <c r="EQ1" t="inlineStr">
+      <c r="EQ1" s="1" t="inlineStr">
         <is>
           <t>Bandwidth Inc. Class A</t>
         </is>
       </c>
-      <c r="ER1" t="inlineStr">
+      <c r="ER1" s="1" t="inlineStr">
         <is>
           <t>Cardlytics, Inc.</t>
         </is>
       </c>
-      <c r="ES1" t="inlineStr">
+      <c r="ES1" s="1" t="inlineStr">
         <is>
           <t>DocuSign, Inc.</t>
         </is>
       </c>
-      <c r="ET1" t="inlineStr">
+      <c r="ET1" s="1" t="inlineStr">
         <is>
           <t>Elastic NV</t>
         </is>
       </c>
-      <c r="EU1" t="inlineStr">
+      <c r="EU1" s="1" t="inlineStr">
         <is>
           <t>Axonics Modulation Technologies, Inc.</t>
         </is>
       </c>
-      <c r="EV1" t="inlineStr">
+      <c r="EV1" s="1" t="inlineStr">
         <is>
           <t>Pinterest, Inc. Class A</t>
         </is>
       </c>
-      <c r="EW1" t="inlineStr">
+      <c r="EW1" s="1" t="inlineStr">
         <is>
           <t>CrowdStrike Holdings, Inc. Class A</t>
         </is>
       </c>
-      <c r="EX1" t="inlineStr">
+      <c r="EX1" s="1" t="inlineStr">
         <is>
           <t>Zoom Video Communications, Inc. Class A</t>
         </is>
       </c>
-      <c r="EY1" t="inlineStr">
+      <c r="EY1" s="1" t="inlineStr">
         <is>
           <t>Uber Technologies, Inc.</t>
         </is>
       </c>
-      <c r="EZ1" t="inlineStr">
+      <c r="EZ1" s="1" t="inlineStr">
         <is>
           <t>Beyond Meat, Inc.</t>
         </is>
       </c>
-      <c r="FA1" t="inlineStr">
+      <c r="FA1" s="1" t="inlineStr">
         <is>
           <t>Fastly, Inc. Class A</t>
         </is>
       </c>
-      <c r="FB1" t="inlineStr">
+      <c r="FB1" s="1" t="inlineStr">
         <is>
           <t>Turning Point Therapeutics, Inc.</t>
         </is>
       </c>
-      <c r="FC1" t="inlineStr">
+      <c r="FC1" s="1" t="inlineStr">
         <is>
           <t>Kodiak Sciences, Inc.</t>
         </is>
       </c>
-      <c r="FD1" t="inlineStr">
+      <c r="FD1" s="1" t="inlineStr">
         <is>
           <t>10x Genomics Inc Class A</t>
         </is>
       </c>
-      <c r="FE1" t="inlineStr">
+      <c r="FE1" s="1" t="inlineStr">
         <is>
           <t>Fiverr International Ltd.</t>
         </is>
       </c>
-      <c r="FF1" t="inlineStr">
+      <c r="FF1" s="1" t="inlineStr">
         <is>
           <t>Phreesia, Inc.</t>
         </is>
       </c>
-      <c r="FG1" t="inlineStr">
+      <c r="FG1" s="1" t="inlineStr">
         <is>
           <t>Sunnova Energy International Inc</t>
         </is>
       </c>
-      <c r="FH1" t="inlineStr">
+      <c r="FH1" s="1" t="inlineStr">
         <is>
           <t>Chewy, Inc. Class A</t>
         </is>
       </c>
-      <c r="FI1" t="inlineStr">
+      <c r="FI1" s="1" t="inlineStr">
         <is>
           <t>Slack Technologies, Inc. Class A</t>
         </is>
       </c>
-      <c r="FJ1" t="inlineStr">
+      <c r="FJ1" s="1" t="inlineStr">
         <is>
           <t>Stoke Therapeutics, Inc.</t>
         </is>
       </c>
-      <c r="FK1" t="inlineStr">
+      <c r="FK1" s="1" t="inlineStr">
         <is>
           <t>Springworks Therapeutics, Inc.</t>
         </is>
       </c>
-      <c r="FL1" t="inlineStr">
+      <c r="FL1" s="1" t="inlineStr">
         <is>
           <t>Cerence Inc.</t>
         </is>
       </c>
-      <c r="FM1" t="inlineStr">
+      <c r="FM1" s="1" t="inlineStr">
         <is>
           <t>IGM Biosciences, Inc.</t>
         </is>
       </c>
-      <c r="FN1" t="inlineStr">
+      <c r="FN1" s="1" t="inlineStr">
         <is>
           <t>Cloudflare Inc Class A</t>
         </is>
       </c>
-      <c r="FO1" t="inlineStr">
+      <c r="FO1" s="1" t="inlineStr">
         <is>
           <t>Peloton Interactive, Inc. Class A</t>
         </is>
       </c>
-      <c r="FP1" t="inlineStr">
+      <c r="FP1" s="1" t="inlineStr">
         <is>
           <t>Datadog Inc Class A</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>2020-01-03</t>
         </is>
@@ -29999,7 +30011,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>2020-01-10</t>
         </is>
@@ -30519,7 +30531,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>2020-01-17</t>
         </is>
@@ -31039,7 +31051,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>2020-01-24</t>
         </is>
@@ -31559,7 +31571,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>2020-01-31</t>
         </is>
@@ -32079,7 +32091,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>2020-02-07</t>
         </is>
@@ -32599,7 +32611,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>2020-02-14</t>
         </is>
@@ -33119,7 +33131,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>2020-02-21</t>
         </is>
@@ -33639,7 +33651,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>2020-02-28</t>
         </is>
@@ -34159,7 +34171,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>2020-03-06</t>
         </is>
@@ -34679,7 +34691,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>2020-03-13</t>
         </is>
@@ -35199,7 +35211,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>2020-03-20</t>
         </is>
@@ -35719,7 +35731,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>2020-03-27</t>
         </is>
@@ -36239,7 +36251,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>2020-04-03</t>
         </is>
@@ -36759,7 +36771,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>2020-04-10</t>
         </is>
@@ -37279,7 +37291,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>2020-04-17</t>
         </is>
@@ -37799,7 +37811,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>2020-04-24</t>
         </is>
@@ -38319,7 +38331,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>2020-05-01</t>
         </is>
@@ -38839,7 +38851,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>2020-05-08</t>
         </is>
@@ -39359,7 +39371,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>2020-05-15</t>
         </is>
@@ -39879,7 +39891,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>2020-05-22</t>
         </is>
@@ -40399,7 +40411,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>2020-05-29</t>
         </is>
@@ -40919,7 +40931,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>2020-06-05</t>
         </is>
@@ -41439,7 +41451,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>2020-06-12</t>
         </is>
@@ -41959,7 +41971,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>2020-06-19</t>
         </is>
@@ -42479,7 +42491,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>2020-06-26</t>
         </is>
@@ -42999,7 +43011,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>2020-07-03</t>
         </is>
@@ -43519,7 +43531,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>2020-07-10</t>
         </is>
@@ -44039,7 +44051,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="1" t="inlineStr">
         <is>
           <t>2020-07-17</t>
         </is>
@@ -44559,7 +44571,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>2020-07-24</t>
         </is>
@@ -45079,7 +45091,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>2020-07-31</t>
         </is>
@@ -45599,7 +45611,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="1" t="inlineStr">
         <is>
           <t>2020-08-07</t>
         </is>
@@ -46119,7 +46131,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="1" t="inlineStr">
         <is>
           <t>2020-08-14</t>
         </is>
@@ -46639,7 +46651,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="1" t="inlineStr">
         <is>
           <t>2020-08-21</t>
         </is>
@@ -47159,7 +47171,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="1" t="inlineStr">
         <is>
           <t>2020-08-28</t>
         </is>
@@ -47679,7 +47691,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="1" t="inlineStr">
         <is>
           <t>2020-09-04</t>
         </is>
@@ -48199,7 +48211,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="1" t="inlineStr">
         <is>
           <t>2020-09-11</t>
         </is>
@@ -48719,7 +48731,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="1" t="inlineStr">
         <is>
           <t>2020-09-18</t>
         </is>
@@ -49239,7 +49251,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="1" t="inlineStr">
         <is>
           <t>2020-09-25</t>
         </is>
@@ -49759,7 +49771,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="1" t="inlineStr">
         <is>
           <t>2020-10-02</t>
         </is>
@@ -50279,7 +50291,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="1" t="inlineStr">
         <is>
           <t>2020-10-09</t>
         </is>
@@ -50799,7 +50811,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="1" t="inlineStr">
         <is>
           <t>2020-10-16</t>
         </is>
@@ -51319,7 +51331,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="1" t="inlineStr">
         <is>
           <t>2020-10-23</t>
         </is>
@@ -51839,7 +51851,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="1" t="inlineStr">
         <is>
           <t>2020-10-30</t>
         </is>
@@ -52359,7 +52371,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="1" t="inlineStr">
         <is>
           <t>2020-11-06</t>
         </is>
@@ -52879,7 +52891,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="1" t="inlineStr">
         <is>
           <t>2020-11-13</t>
         </is>
@@ -53399,7 +53411,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="1" t="inlineStr">
         <is>
           <t>2020-11-20</t>
         </is>
@@ -53919,7 +53931,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="1" t="inlineStr">
         <is>
           <t>2020-11-27</t>
         </is>
@@ -54439,7 +54451,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="1" t="inlineStr">
         <is>
           <t>2020-12-04</t>
         </is>
@@ -54959,7 +54971,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="1" t="inlineStr">
         <is>
           <t>2020-12-11</t>
         </is>
@@ -55479,7 +55491,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="1" t="inlineStr">
         <is>
           <t>2020-12-18</t>
         </is>
@@ -55999,7 +56011,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="1" t="inlineStr">
         <is>
           <t>2020-12-25</t>
         </is>

</xml_diff>